<commit_message>
starting figuring out data
</commit_message>
<xml_diff>
--- a/raw_data/tableMaster.xlsx
+++ b/raw_data/tableMaster.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anhqu\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anhqu\OneDrive\Documents\JobProjection\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47B4386-546F-48A9-A60F-348A775DDA0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A460354-861E-4519-9671-77C25000E803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0B945E46-D09C-4793-AFE9-C8D9EC28E047}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
   <si>
     <t>Sheet Name</t>
   </si>
@@ -117,6 +117,15 @@
   </si>
   <si>
     <t>Median earnings per degree</t>
+  </si>
+  <si>
+    <t>Everything</t>
+  </si>
+  <si>
+    <t>Dashboard/data viz</t>
+  </si>
+  <si>
+    <t>There are misisng data</t>
   </si>
 </sst>
 </file>
@@ -175,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -189,9 +198,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -536,7 +542,7 @@
     <col min="4" max="4" width="14.6328125" customWidth="1"/>
     <col min="5" max="5" width="18.54296875" customWidth="1"/>
     <col min="6" max="6" width="22.1796875" customWidth="1"/>
-    <col min="7" max="7" width="27.1796875" style="6" customWidth="1"/>
+    <col min="7" max="7" width="27.1796875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -569,6 +575,18 @@
       <c r="B2" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="3" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
@@ -577,6 +595,18 @@
       <c r="B3" s="2" t="s">
         <v>16</v>
       </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
@@ -585,6 +615,18 @@
       <c r="B4" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
@@ -593,6 +635,18 @@
       <c r="B5" s="2" t="s">
         <v>18</v>
       </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="6" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
@@ -609,7 +663,7 @@
       <c r="B7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -617,7 +671,7 @@
       <c r="A8" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D8">
@@ -628,7 +682,7 @@
       <c r="A9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="2" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>